<commit_message>
Fix sign-in log timezone: convert UTC to IST (UTC+5:30)
</commit_message>
<xml_diff>
--- a/Sign_In_Log.xlsx
+++ b/Sign_In_Log.xlsx
@@ -512,7 +512,7 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated on: 22 September 2026, 10:24 PM</t>
+          <t>Generated on: 22 September 2026, 10:36 PM</t>
         </is>
       </c>
     </row>
@@ -589,7 +589,7 @@
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>12:29:16 PM</t>
+          <t>05:59:16 PM</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr">
@@ -629,7 +629,7 @@
       </c>
       <c r="G6" s="6" t="inlineStr">
         <is>
-          <t>12:35:36 PM</t>
+          <t>06:05:36 PM</t>
         </is>
       </c>
       <c r="H6" s="6" t="inlineStr">
@@ -669,7 +669,7 @@
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>12:52:07 PM</t>
+          <t>06:22:07 PM</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
@@ -709,7 +709,7 @@
       </c>
       <c r="G8" s="6" t="inlineStr">
         <is>
-          <t>03:57:57 PM</t>
+          <t>09:27:57 PM</t>
         </is>
       </c>
       <c r="H8" s="6" t="inlineStr">

</xml_diff>